<commit_message>
Uppdaterat verksamhetsdata från Excel
</commit_message>
<xml_diff>
--- a/data/source/2026/events_master.xlsx
+++ b/data/source/2026/events_master.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alk/Desktop/Utredare/Cykler/interactive/verksamhetscykel/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alk/Desktop/HDa/Styrning/System/Del av cykel/Verksamhetscykel/interactive/verksamhetscykel/data/source/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89AB43B6-9D9F-8F46-9939-5702BEEAEF07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D23386D-4CDF-3442-97D0-425E6C0F15C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Verksamhetscykel" sheetId="1" r:id="rId1"/>
@@ -460,26 +460,6 @@
     <dxf>
       <font>
         <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="yyyy/mm/dd"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -586,6 +566,26 @@
         </patternFill>
       </fill>
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="yyyy/mm/dd"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -831,12 +831,12 @@
     <tableColumn id="13" xr3:uid="{AE550A58-E5ED-084C-9C14-4A2C188A5604}" name="Styrningsunderlag förkortning" dataDxfId="8"/>
     <tableColumn id="11" xr3:uid="{D15A5E67-83CD-5444-833F-E228EFC07424}" name="Verksamhet" dataDxfId="7"/>
     <tableColumn id="14" xr3:uid="{B30DBDC3-BAA7-1E44-832A-A3CEF8C37C40}" name="Ekonomi" dataDxfId="6"/>
-    <tableColumn id="1" xr3:uid="{9E30171B-BE3F-6340-8BE1-11D1891834E8}" name="Kvalitét" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{0E4B8298-FBDD-164C-A965-14897F288509}" name="Styrningsfas" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{268E9011-16AB-6B44-BEF8-3B79865B9ABD}" name="Relaterad styrningsfas" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{FE25B613-BB4D-BE48-8565-29261E506D49}" name="Typ" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{E8BD3A96-2661-B44D-A4D7-370417830062}" name="Ansvarig" dataDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{7FD3B4E7-838B-644D-9C26-F6AE5C7FA71B}" name="Synlig" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{9E30171B-BE3F-6340-8BE1-11D1891834E8}" name="Kvalitét" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{0E4B8298-FBDD-164C-A965-14897F288509}" name="Styrningsfas" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{268E9011-16AB-6B44-BEF8-3B79865B9ABD}" name="Relaterad styrningsfas" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{FE25B613-BB4D-BE48-8565-29261E506D49}" name="Typ" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{E8BD3A96-2661-B44D-A4D7-370417830062}" name="Ansvarig" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{7FD3B4E7-838B-644D-9C26-F6AE5C7FA71B}" name="Synlig" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1130,7 +1130,7 @@
   <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.5" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42.83203125" customWidth="1"/>
     <col min="4" max="4" width="35.83203125" customWidth="1"/>
@@ -1676,10 +1676,10 @@
     </row>
     <row r="16" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="13">
-        <v>46157</v>
+        <v>46346</v>
       </c>
       <c r="B16" s="13">
-        <v>46157</v>
+        <v>46346</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>7</v>

</xml_diff>